<commit_message>
PROSANITAS - AUTOLABNET - 1.1: TestCase RAD #2
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#PROSANITASSRLXX/PROSANITASSRL/AUTOLABNET/1.1/report-checklist.xlsx
+++ b/GATEWAY/A1#111#PROSANITASSRLXX/PROSANITASSRL/AUTOLABNET/1.1/report-checklist.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\git_fse\it-fse-accreditamento\GATEWAY\A1#111#PROSANITASSRLXX\PROSANITAS_SRL\AUTOLABNET\1.1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitAtWork\LabTBM.FSE\A1#111#PROSANITASSRLXX\PROSANITAS_SRL\AUTOLABNET\1.1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B915ECEC-84FD-445B-9FF6-A72BF5C51A61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14FE393F-9FC0-4963-B365-DA4FD169F13C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-32670" yWindow="930" windowWidth="21600" windowHeight="12900" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="435" yWindow="120" windowWidth="25500" windowHeight="11595" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Istruzioni Compilazione" sheetId="1" r:id="rId1"/>
@@ -83,7 +83,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="211">
   <si>
     <t>COME VALORIZZARE LA CHECKLIST (tab TestCases)</t>
   </si>
@@ -889,6 +889,9 @@
   </si>
   <si>
     <t>a085a97ae7d576851d4ff0d31839cd5e</t>
+  </si>
+  <si>
+    <t>"INVIO FSE NON RIUSCITO: errore di connessione, verificare"</t>
   </si>
 </sst>
 </file>
@@ -3267,12 +3270,24 @@
       <c r="K10" s="35"/>
       <c r="L10" s="35"/>
       <c r="M10" s="35"/>
-      <c r="N10" s="35"/>
-      <c r="O10" s="35"/>
-      <c r="P10" s="35"/>
-      <c r="Q10" s="35"/>
-      <c r="R10" s="35"/>
-      <c r="S10" s="35"/>
+      <c r="N10" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="O10" s="35" t="s">
+        <v>210</v>
+      </c>
+      <c r="P10" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q10" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="R10" s="35" t="s">
+        <v>80</v>
+      </c>
+      <c r="S10" s="35" t="s">
+        <v>149</v>
+      </c>
       <c r="T10" s="35"/>
       <c r="U10" s="36"/>
       <c r="V10" s="37"/>
@@ -3314,12 +3329,24 @@
       <c r="K11" s="35"/>
       <c r="L11" s="35"/>
       <c r="M11" s="35"/>
-      <c r="N11" s="35"/>
-      <c r="O11" s="35"/>
-      <c r="P11" s="35"/>
-      <c r="Q11" s="35"/>
-      <c r="R11" s="35"/>
-      <c r="S11" s="35"/>
+      <c r="N11" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="O11" s="35" t="s">
+        <v>210</v>
+      </c>
+      <c r="P11" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q11" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="R11" s="35" t="s">
+        <v>80</v>
+      </c>
+      <c r="S11" s="35" t="s">
+        <v>149</v>
+      </c>
       <c r="T11" s="35"/>
       <c r="U11" s="36"/>
       <c r="V11" s="37"/>
@@ -10603,6 +10630,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100BE9A258ADBC3EC4CBEB1E2AB9909207A" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="0284f501378927579289f00316ec8a74">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="295b7897-c886-40bf-9750-5782b814c3e4" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b47213d65be806e283915cff374a7eef" ns2:_="">
     <xsd:import namespace="295b7897-c886-40bf-9750-5782b814c3e4"/>
@@ -10746,22 +10788,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C4C806F-EC4E-4231-9462-6D32094C4603}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7568E770-0BC4-46AF-B6C6-958AE21C8F7F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -10779,31 +10831,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C4C806F-EC4E-4231-9462-6D32094C4603}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{e0793d39-0939-496d-b129-198edd916feb}" enabled="0" method="" siteId="{e0793d39-0939-496d-b129-198edd916feb}" removed="1"/>

</xml_diff>

<commit_message>
PROSANITASSRL#AUTOLABNET#1.1 : fix su TC_25 (471), TC_26 (472) e TC_27 (474)
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#PROSANITASSRLXX/PROSANITASSRL/AUTOLABNET/1.1/report-checklist.xlsx
+++ b/GATEWAY/A1#111#PROSANITASSRLXX/PROSANITASSRL/AUTOLABNET/1.1/report-checklist.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\robyr\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\git_fse\klaus-it-fse-accreditamento\GATEWAY\A1#111#PROSANITASSRLXX\PROSANITASSRL\AUTOLABNET\1.1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9416920B-D5D9-4A0A-B63E-005505CEE86F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA0AB018-A1A6-49FC-919E-0F31F432B735}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2115" yWindow="690" windowWidth="25500" windowHeight="11595" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Istruzioni Compilazione" sheetId="1" r:id="rId1"/>
@@ -846,33 +846,6 @@
     <t>2.16.840.1.113883.2.9.2.120.4.4.82a1bcb3ceea777f60fd153f6ec968824d48cbdd877242dfde81a97ed7d9e51f.29c13e19fe^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
-    <t>a3d67b4395a01d23d25d10beafe9cbb8</t>
-  </si>
-  <si>
-    <t>2026-02-22T23:40:02Z</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.82a1bcb3ceea777f60fd153f6ec968824d48cbdd877242dfde81a97ed7d9e51f.c59626a854^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>62fb70fb350322be5421d976a4bfb660</t>
-  </si>
-  <si>
-    <t>2026-02-22T22:48:18Z</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.82a1bcb3ceea777f60fd153f6ec968824d48cbdd877242dfde81a97ed7d9e51f.1a5f0894b2^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>2026-02-23T12:18:29Z</t>
-  </si>
-  <si>
-    <t>38b645be8a2c2cb4324e905a43dda514</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.82a1bcb3ceea777f60fd153f6ec968824d48cbdd877242dfde81a97ed7d9e51f.14b1e1f3d9^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
     <t>"INVIO FSE NON RIUSCITO: endpoint non raggiungibile"</t>
   </si>
   <si>
@@ -892,6 +865,33 @@
   </si>
   <si>
     <t>"INVIO FSE NON RIUSCITO: errore di connessione, verificare"</t>
+  </si>
+  <si>
+    <t>2026-03-28T07:49:00Z</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.82a1bcb3ceea777f60fd153f6ec968824d48cbdd877242dfde81a97ed7d9e51f.9296f2015e^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2b1a652a61b698dde7e2dc6af44e4976</t>
+  </si>
+  <si>
+    <t>2026-03-28T07:49:40Z</t>
+  </si>
+  <si>
+    <t>4bb209b3ae277d4c8d33095ca432d153</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.82a1bcb3ceea777f60fd153f6ec968824d48cbdd877242dfde81a97ed7d9e51f.4d44f388a4^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>ffdc4a172c078ebe404684ac753842c1</t>
+  </si>
+  <si>
+    <t>2026-03-28T07:52:38Z</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.82a1bcb3ceea777f60fd153f6ec968824d48cbdd877242dfde81a97ed7d9e51f.ee44a54cbf^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
 </sst>
 </file>
@@ -3256,13 +3256,13 @@
         <v>46077</v>
       </c>
       <c r="G10" s="34" t="s">
-        <v>208</v>
+        <v>199</v>
       </c>
       <c r="H10" s="34" t="s">
-        <v>209</v>
+        <v>200</v>
       </c>
       <c r="I10" s="39" t="s">
-        <v>207</v>
+        <v>198</v>
       </c>
       <c r="J10" s="35" t="s">
         <v>49</v>
@@ -3276,7 +3276,7 @@
         <v>49</v>
       </c>
       <c r="O10" s="35" t="s">
-        <v>210</v>
+        <v>201</v>
       </c>
       <c r="P10" s="35" t="s">
         <v>49</v>
@@ -3317,13 +3317,13 @@
         <v>46077</v>
       </c>
       <c r="G11" s="34" t="s">
-        <v>205</v>
+        <v>196</v>
       </c>
       <c r="H11" s="34" t="s">
-        <v>206</v>
+        <v>197</v>
       </c>
       <c r="I11" s="39" t="s">
-        <v>207</v>
+        <v>198</v>
       </c>
       <c r="J11" s="35" t="s">
         <v>49</v>
@@ -3337,7 +3337,7 @@
         <v>49</v>
       </c>
       <c r="O11" s="35" t="s">
-        <v>210</v>
+        <v>201</v>
       </c>
       <c r="P11" s="35" t="s">
         <v>49</v>
@@ -3394,7 +3394,7 @@
         <v>49</v>
       </c>
       <c r="O12" s="35" t="s">
-        <v>204</v>
+        <v>195</v>
       </c>
       <c r="P12" s="35" t="s">
         <v>49</v>
@@ -4449,16 +4449,16 @@
         <v>124</v>
       </c>
       <c r="F30" s="34">
-        <v>46076</v>
+        <v>46109</v>
       </c>
       <c r="G30" s="34" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="H30" s="34" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="I30" s="39" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="J30" s="35" t="s">
         <v>49</v>
@@ -4496,16 +4496,16 @@
         <v>126</v>
       </c>
       <c r="F31" s="34">
-        <v>46076</v>
+        <v>46109</v>
       </c>
       <c r="G31" s="34" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="H31" s="34" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="I31" s="39" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="J31" s="35" t="s">
         <v>49</v>
@@ -4543,16 +4543,16 @@
         <v>129</v>
       </c>
       <c r="F32" s="34">
-        <v>46076</v>
+        <v>46109</v>
       </c>
       <c r="G32" s="34" t="s">
-        <v>196</v>
+        <v>209</v>
       </c>
       <c r="H32" s="34" t="s">
-        <v>195</v>
+        <v>208</v>
       </c>
       <c r="I32" s="39" t="s">
-        <v>197</v>
+        <v>210</v>
       </c>
       <c r="J32" s="35" t="s">
         <v>49</v>
@@ -10634,21 +10634,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100BE9A258ADBC3EC4CBEB1E2AB9909207A" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="0284f501378927579289f00316ec8a74">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="295b7897-c886-40bf-9750-5782b814c3e4" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b47213d65be806e283915cff374a7eef" ns2:_="">
     <xsd:import namespace="295b7897-c886-40bf-9750-5782b814c3e4"/>
@@ -10792,10 +10777,35 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7568E770-0BC4-46AF-B6C6-958AE21C8F7F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="295b7897-c886-40bf-9750-5782b814c3e4"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -10818,19 +10828,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7568E770-0BC4-46AF-B6C6-958AE21C8F7F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="295b7897-c886-40bf-9750-5782b814c3e4"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>